<commit_message>
Bug Fix: Question display(Time) & Button Display(Home)
</commit_message>
<xml_diff>
--- a/MathTutor/questions/question.xlsx
+++ b/MathTutor/questions/question.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="68">
   <si>
     <t xml:space="preserve">question</t>
   </si>
@@ -152,9 +152,6 @@
   </si>
   <si>
     <t xml:space="preserve">a1:10*b1:10*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">{a}*+b}</t>
   </si>
   <si>
     <t xml:space="preserve">{a} % of {b} =</t>
@@ -347,7 +344,7 @@
   <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.4" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="107.28"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="42.89"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.55"/>
   </cols>
@@ -646,7 +643,7 @@
         <v>1</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>44</v>
+        <v>22</v>
       </c>
       <c r="F15" s="0" t="n">
         <v>5</v>
@@ -654,19 +651,19 @@
     </row>
     <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="B16" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="C16" s="0" t="s">
         <v>46</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>47</v>
       </c>
       <c r="D16" s="0" t="n">
         <v>2</v>
       </c>
       <c r="E16" s="0" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F16" s="0" t="n">
         <v>5</v>
@@ -674,19 +671,19 @@
     </row>
     <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
+        <v>44</v>
+      </c>
+      <c r="B17" s="0" t="s">
         <v>45</v>
       </c>
-      <c r="B17" s="0" t="s">
-        <v>46</v>
-      </c>
       <c r="C17" s="0" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D17" s="0" t="n">
         <v>3</v>
       </c>
       <c r="E17" s="0" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F17" s="0" t="n">
         <v>10</v>
@@ -700,7 +697,7 @@
         <v>40</v>
       </c>
       <c r="C18" s="0" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D18" s="0" t="n">
         <v>2</v>
@@ -720,7 +717,7 @@
         <v>40</v>
       </c>
       <c r="C19" s="0" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D19" s="0" t="n">
         <v>3</v>
@@ -734,19 +731,19 @@
     </row>
     <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="C20" s="0" t="s">
         <v>53</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="D20" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" s="0" t="s">
         <v>54</v>
-      </c>
-      <c r="D20" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E20" s="0" t="s">
-        <v>55</v>
       </c>
       <c r="F20" s="0" t="n">
         <v>5</v>
@@ -754,19 +751,19 @@
     </row>
     <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B21" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="B21" s="0" t="s">
-        <v>53</v>
-      </c>
       <c r="C21" s="0" t="s">
+        <v>55</v>
+      </c>
+      <c r="D21" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="0" t="s">
         <v>56</v>
-      </c>
-      <c r="D21" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E21" s="0" t="s">
-        <v>57</v>
       </c>
       <c r="F21" s="0" t="n">
         <v>5</v>
@@ -774,19 +771,19 @@
     </row>
     <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B22" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="B22" s="0" t="s">
-        <v>53</v>
-      </c>
       <c r="C22" s="0" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D22" s="0" t="n">
         <v>2</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F22" s="0" t="n">
         <v>7</v>
@@ -794,19 +791,19 @@
     </row>
     <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="0" t="s">
         <v>52</v>
       </c>
-      <c r="B23" s="0" t="s">
-        <v>53</v>
-      </c>
       <c r="C23" s="0" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D23" s="0" t="n">
         <v>2</v>
       </c>
       <c r="E23" s="0" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F23" s="0" t="n">
         <v>7</v>
@@ -814,19 +811,19 @@
     </row>
     <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="C24" s="0" t="s">
         <v>60</v>
       </c>
-      <c r="B24" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="C24" s="0" t="s">
+      <c r="D24" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="0" t="s">
         <v>61</v>
-      </c>
-      <c r="D24" s="0" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="0" t="s">
-        <v>62</v>
       </c>
       <c r="F24" s="0" t="n">
         <v>7</v>
@@ -834,19 +831,19 @@
     </row>
     <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B25" s="0" t="s">
         <v>40</v>
       </c>
       <c r="C25" s="0" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D25" s="0" t="n">
         <v>2</v>
       </c>
       <c r="E25" s="0" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F25" s="0" t="n">
         <v>10</v>
@@ -854,10 +851,10 @@
     </row>
     <row r="26" customFormat="false" ht="14.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
+        <v>65</v>
+      </c>
+      <c r="B26" s="0" t="s">
         <v>66</v>
-      </c>
-      <c r="B26" s="0" t="s">
-        <v>67</v>
       </c>
       <c r="C26" s="0" t="s">
         <v>43</v>
@@ -866,7 +863,7 @@
         <v>1</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F26" s="0" t="n">
         <v>10</v>
@@ -875,8 +872,8 @@
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>